<commit_message>
Consenti venditori affidatari esterni
</commit_message>
<xml_diff>
--- a/calottino_categoria_gestione.xlsx
+++ b/calottino_categoria_gestione.xlsx
@@ -2,16 +2,17 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0d6326f5f2c34ca5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istruzioni" sheetId="2" r:id="R4530ee0cbbf24d38"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parametri" sheetId="3" r:id="R3b945633529a4b05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persone_Quote" sheetId="4" r:id="R125d03550e6d4ccc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisti_Patch" sheetId="5" r:id="R4550e452985c4ae8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendite_Patch" sheetId="6" r:id="R534ab63ffae54b76"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spese_Categoria" sheetId="7" r:id="Rbae4cfaf1ffc4b75"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Magazzino_Cassa" sheetId="8" r:id="Ra7d8da550e41432c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liste" sheetId="9" r:id="R920da7b190a4415a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Affidamenti_Patch" sheetId="10" r:id="R862f6891bd0b4e69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="Ra25f54df89444676"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Istruzioni" sheetId="2" r:id="Rc24f2c3c8ebd4ab2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parametri" sheetId="3" r:id="R10128236b66f45b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Persone_Quote" sheetId="4" r:id="R89538b0c07a943e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Acquisti_Patch" sheetId="5" r:id="Ra63aa00fcbe04517"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendite_Patch" sheetId="6" r:id="Rdc8652a562ad482c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spese_Categoria" sheetId="7" r:id="R81d3810f50a14c3c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Magazzino_Cassa" sheetId="8" r:id="R75a21954f5cb4865"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liste" sheetId="9" r:id="Rba124f79ade74446"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Affidamenti_Patch" sheetId="10" r:id="Rba0df0b5f7774190"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venditori_Affidatari" sheetId="11" r:id="Rf85801af9e494c09"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -633,7 +634,7 @@
     <x:numFmt numFmtId="167" formatCode="0.0%"/>
     <x:numFmt numFmtId="200" formatCode="#,##0"/>
   </x:numFmts>
-  <x:fonts count="15">
+  <x:fonts count="16">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -716,8 +717,14 @@
       <x:color rgb="FF111827"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="10">
+  <x:fills count="14">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -762,6 +769,26 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDBEAFE"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F766E"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF7ED"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -861,7 +888,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="76">
+  <x:cellXfs count="94">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1047,6 +1074,48 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="11" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="15" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="15" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="13" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="13" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="13" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="13" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="13" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -1873,7 +1942,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R8ed3830dcf534dbf"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Reeb5144390e04c66"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -1908,7 +1977,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R76b70b901cb449ef"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rf3df260e30a14f94"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2009,6 +2078,17 @@
     <x:tableColumn id="8" name="Versato in cassa"/>
     <x:tableColumn id="9" name="Denaro da versare"/>
     <x:tableColumn id="10" name="Stato / Note"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TabellaVenditoriAffidatari" displayName="TabellaVenditoriAffidatari" ref="A3:C103" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="3">
+    <x:tableColumn id="1" name="Tipo"/>
+    <x:tableColumn id="2" name="Nome / Cognome"/>
+    <x:tableColumn id="3" name="Note"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -2638,7 +2718,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R155fbdaf98ff40d7"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5c1f14340e14e9c"/>
 </x:worksheet>
 </file>
 
@@ -6729,7 +6809,7 @@
       <x:formula2>2100-12-31</x:formula2>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="B4:B203">
-      <x:formula1>'Persone_Quote'!$B$4:$B$18</x:formula1>
+      <x:formula1>'Venditori_Affidatari'!$B$4:$B$103</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="whole" operator="greaterThanOrEqual" sqref="C4:C203">
       <x:formula1>0</x:formula1>
@@ -6743,7 +6823,828 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R50a70dec9ab64fe8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7c1dcd57791c4a2f"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="27" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="40" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="27" customHeight="1">
+      <x:c r="A1" s="78" t="str">
+        <x:v>Elenco venditori affidatari</x:v>
+      </x:c>
+      <x:c r="B1" s="78"/>
+      <x:c r="C1" s="78"/>
+    </x:row>
+    <x:row r="2" ht="38" customHeight="1">
+      <x:c r="A2" s="82" t="str">
+        <x:v>I componenti sono riportati automaticamente. Per aggiungere colleghi o amici, scrivi il loro nome nelle righe della sezione Esterni.</x:v>
+      </x:c>
+      <x:c r="B2" s="82"/>
+      <x:c r="C2" s="82"/>
+    </x:row>
+    <x:row r="3" ht="28" customHeight="1">
+      <x:c r="A3" s="87" t="str">
+        <x:v>Tipo</x:v>
+      </x:c>
+      <x:c r="B3" s="87" t="str">
+        <x:v>Nome / Cognome</x:v>
+      </x:c>
+      <x:c r="C3" s="87" t="str">
+        <x:v>Note</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="22" customHeight="1">
+      <x:c r="A4" s="55" t="str">
+        <x:v>Componente</x:v>
+      </x:c>
+      <x:c r="B4" s="56" t="str">
+        <x:f>'Persone_Quote'!B4</x:f>
+        <x:v>Capodanno</x:v>
+      </x:c>
+      <x:c r="C4" s="57" t="str">
+        <x:v>Elenco automatico dei componenti</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="22" customHeight="1">
+      <x:c r="A5" s="58" t="str">
+        <x:v>Componente</x:v>
+      </x:c>
+      <x:c r="B5" s="59" t="str">
+        <x:f>'Persone_Quote'!B5</x:f>
+        <x:v>Caggia</x:v>
+      </x:c>
+      <x:c r="C5" s="60" t="str">
+        <x:v>Elenco automatico dei componenti</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="22" customHeight="1">
+      <x:c r="A6" s="58" t="str">
+        <x:v>Componente</x:v>
+      </x:c>
+      <x:c r="B6" s="59" t="str">
+        <x:f>'Persone_Quote'!B6</x:f>
+        <x:v>Marchesani</x:v>
+      </x:c>
+      <x:c r="C6" s="60" t="str">
+        <x:v>Elenco automatico dei componenti</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="22" customHeight="1">
+      <x:c r="A7" s="58" t="str">
+        <x:v>Componente</x:v>
+      </x:c>
+      <x:c r="B7" s="59" t="str">
+        <x:f>'Persone_Quote'!B7</x:f>
+        <x:v>Zubenko</x:v>
+      </x:c>
+      <x:c r="C7" s="60" t="str">
+        <x:v>Elenco automatico dei componenti</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="22" customHeight="1">
+      <x:c r="A8" s="58" t="str">
+        <x:v>Componente</x:v>
+      </x:c>
+      <x:c r="B8" s="59" t="str">
+        <x:f>'Persone_Quote'!B8</x:f>
+        <x:v>Losito</x:v>
+      </x:c>
+      <x:c r="C8" s="60" t="str">
+        <x:v>Elenco automatico dei componenti</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="22" customHeight="1">
+      <x:c r="A9" s="58" t="str">
+        <x:v>Componente</x:v>
+      </x:c>
+      <x:c r="B9" s="59" t="str">
+        <x:f>'Persone_Quote'!B9</x:f>
+        <x:v>Di Stefano</x:v>
+      </x:c>
+      <x:c r="C9" s="60" t="str">
+        <x:v>Elenco automatico dei componenti</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="22" customHeight="1">
+      <x:c r="A10" s="58" t="str">
+        <x:v>Componente</x:v>
+      </x:c>
+      <x:c r="B10" s="59" t="str">
+        <x:f>'Persone_Quote'!B10</x:f>
+        <x:v>Palladino</x:v>
+      </x:c>
+      <x:c r="C10" s="60" t="str">
+        <x:v>Elenco automatico dei componenti</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="22" customHeight="1">
+      <x:c r="A11" s="58" t="str">
+        <x:v>Componente</x:v>
+      </x:c>
+      <x:c r="B11" s="59" t="str">
+        <x:f>'Persone_Quote'!B11</x:f>
+        <x:v>Locorotondo</x:v>
+      </x:c>
+      <x:c r="C11" s="60" t="str">
+        <x:v>Elenco automatico dei componenti</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="22" customHeight="1">
+      <x:c r="A12" s="58" t="str">
+        <x:v>Componente</x:v>
+      </x:c>
+      <x:c r="B12" s="59" t="str">
+        <x:f>'Persone_Quote'!B12</x:f>
+        <x:v>Pertosa</x:v>
+      </x:c>
+      <x:c r="C12" s="60" t="str">
+        <x:v>Elenco automatico dei componenti</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="22" customHeight="1">
+      <x:c r="A13" s="58" t="str">
+        <x:v>Componente</x:v>
+      </x:c>
+      <x:c r="B13" s="59" t="str">
+        <x:f>'Persone_Quote'!B13</x:f>
+        <x:v>Ottaiano</x:v>
+      </x:c>
+      <x:c r="C13" s="60" t="str">
+        <x:v>Elenco automatico dei componenti</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="22" customHeight="1">
+      <x:c r="A14" s="58" t="str">
+        <x:v>Componente</x:v>
+      </x:c>
+      <x:c r="B14" s="59" t="str">
+        <x:f>'Persone_Quote'!B14</x:f>
+        <x:v>Fragnito</x:v>
+      </x:c>
+      <x:c r="C14" s="60" t="str">
+        <x:v>Elenco automatico dei componenti</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="22" customHeight="1">
+      <x:c r="A15" s="58" t="str">
+        <x:v>Componente</x:v>
+      </x:c>
+      <x:c r="B15" s="59" t="str">
+        <x:f>'Persone_Quote'!B15</x:f>
+        <x:v>Murolo</x:v>
+      </x:c>
+      <x:c r="C15" s="60" t="str">
+        <x:v>Elenco automatico dei componenti</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="22" customHeight="1">
+      <x:c r="A16" s="58" t="str">
+        <x:v>Componente</x:v>
+      </x:c>
+      <x:c r="B16" s="59" t="str">
+        <x:f>'Persone_Quote'!B16</x:f>
+        <x:v>Palma</x:v>
+      </x:c>
+      <x:c r="C16" s="60" t="str">
+        <x:v>Elenco automatico dei componenti</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="22" customHeight="1">
+      <x:c r="A17" s="58" t="str">
+        <x:v>Componente</x:v>
+      </x:c>
+      <x:c r="B17" s="59" t="str">
+        <x:f>'Persone_Quote'!B17</x:f>
+        <x:v>Babele</x:v>
+      </x:c>
+      <x:c r="C17" s="60" t="str">
+        <x:v>Elenco automatico dei componenti</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="22" customHeight="1">
+      <x:c r="A18" s="58" t="str">
+        <x:v>Componente</x:v>
+      </x:c>
+      <x:c r="B18" s="59" t="str">
+        <x:f>'Persone_Quote'!B18</x:f>
+        <x:v>Torrente</x:v>
+      </x:c>
+      <x:c r="C18" s="60" t="str">
+        <x:v>Elenco automatico dei componenti</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="22" customHeight="1">
+      <x:c r="A19" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B19" s="89"/>
+      <x:c r="C19" s="90"/>
+    </x:row>
+    <x:row r="20" ht="22" customHeight="1">
+      <x:c r="A20" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B20" s="89"/>
+      <x:c r="C20" s="90"/>
+    </x:row>
+    <x:row r="21" ht="22" customHeight="1">
+      <x:c r="A21" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B21" s="89"/>
+      <x:c r="C21" s="90"/>
+    </x:row>
+    <x:row r="22" ht="22" customHeight="1">
+      <x:c r="A22" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B22" s="89"/>
+      <x:c r="C22" s="90"/>
+    </x:row>
+    <x:row r="23" ht="22" customHeight="1">
+      <x:c r="A23" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B23" s="89"/>
+      <x:c r="C23" s="90"/>
+    </x:row>
+    <x:row r="24" ht="22" customHeight="1">
+      <x:c r="A24" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B24" s="89"/>
+      <x:c r="C24" s="90"/>
+    </x:row>
+    <x:row r="25" ht="22" customHeight="1">
+      <x:c r="A25" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B25" s="89"/>
+      <x:c r="C25" s="90"/>
+    </x:row>
+    <x:row r="26" ht="22" customHeight="1">
+      <x:c r="A26" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B26" s="89"/>
+      <x:c r="C26" s="90"/>
+    </x:row>
+    <x:row r="27" ht="22" customHeight="1">
+      <x:c r="A27" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B27" s="89"/>
+      <x:c r="C27" s="90"/>
+    </x:row>
+    <x:row r="28" ht="22" customHeight="1">
+      <x:c r="A28" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B28" s="89"/>
+      <x:c r="C28" s="90"/>
+    </x:row>
+    <x:row r="29" ht="22" customHeight="1">
+      <x:c r="A29" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B29" s="89"/>
+      <x:c r="C29" s="90"/>
+    </x:row>
+    <x:row r="30" ht="22" customHeight="1">
+      <x:c r="A30" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B30" s="89"/>
+      <x:c r="C30" s="90"/>
+    </x:row>
+    <x:row r="31" ht="22" customHeight="1">
+      <x:c r="A31" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B31" s="89"/>
+      <x:c r="C31" s="90"/>
+    </x:row>
+    <x:row r="32" ht="22" customHeight="1">
+      <x:c r="A32" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B32" s="89"/>
+      <x:c r="C32" s="90"/>
+    </x:row>
+    <x:row r="33" ht="22" customHeight="1">
+      <x:c r="A33" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B33" s="89"/>
+      <x:c r="C33" s="90"/>
+    </x:row>
+    <x:row r="34" ht="22" customHeight="1">
+      <x:c r="A34" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B34" s="89"/>
+      <x:c r="C34" s="90"/>
+    </x:row>
+    <x:row r="35" ht="22" customHeight="1">
+      <x:c r="A35" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B35" s="89"/>
+      <x:c r="C35" s="90"/>
+    </x:row>
+    <x:row r="36" ht="22" customHeight="1">
+      <x:c r="A36" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B36" s="89"/>
+      <x:c r="C36" s="90"/>
+    </x:row>
+    <x:row r="37" ht="22" customHeight="1">
+      <x:c r="A37" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B37" s="89"/>
+      <x:c r="C37" s="90"/>
+    </x:row>
+    <x:row r="38" ht="22" customHeight="1">
+      <x:c r="A38" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B38" s="89"/>
+      <x:c r="C38" s="90"/>
+    </x:row>
+    <x:row r="39" ht="22" customHeight="1">
+      <x:c r="A39" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B39" s="89"/>
+      <x:c r="C39" s="90"/>
+    </x:row>
+    <x:row r="40" ht="22" customHeight="1">
+      <x:c r="A40" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B40" s="89"/>
+      <x:c r="C40" s="90"/>
+    </x:row>
+    <x:row r="41" ht="22" customHeight="1">
+      <x:c r="A41" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B41" s="89"/>
+      <x:c r="C41" s="90"/>
+    </x:row>
+    <x:row r="42" ht="22" customHeight="1">
+      <x:c r="A42" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B42" s="89"/>
+      <x:c r="C42" s="90"/>
+    </x:row>
+    <x:row r="43" ht="22" customHeight="1">
+      <x:c r="A43" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B43" s="89"/>
+      <x:c r="C43" s="90"/>
+    </x:row>
+    <x:row r="44" ht="22" customHeight="1">
+      <x:c r="A44" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B44" s="89"/>
+      <x:c r="C44" s="90"/>
+    </x:row>
+    <x:row r="45" ht="22" customHeight="1">
+      <x:c r="A45" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B45" s="89"/>
+      <x:c r="C45" s="90"/>
+    </x:row>
+    <x:row r="46" ht="22" customHeight="1">
+      <x:c r="A46" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B46" s="89"/>
+      <x:c r="C46" s="90"/>
+    </x:row>
+    <x:row r="47" ht="22" customHeight="1">
+      <x:c r="A47" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B47" s="89"/>
+      <x:c r="C47" s="90"/>
+    </x:row>
+    <x:row r="48" ht="22" customHeight="1">
+      <x:c r="A48" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B48" s="89"/>
+      <x:c r="C48" s="90"/>
+    </x:row>
+    <x:row r="49" ht="22" customHeight="1">
+      <x:c r="A49" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B49" s="89"/>
+      <x:c r="C49" s="90"/>
+    </x:row>
+    <x:row r="50" ht="22" customHeight="1">
+      <x:c r="A50" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B50" s="89"/>
+      <x:c r="C50" s="90"/>
+    </x:row>
+    <x:row r="51" ht="22" customHeight="1">
+      <x:c r="A51" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B51" s="89"/>
+      <x:c r="C51" s="90"/>
+    </x:row>
+    <x:row r="52" ht="22" customHeight="1">
+      <x:c r="A52" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B52" s="89"/>
+      <x:c r="C52" s="90"/>
+    </x:row>
+    <x:row r="53" ht="22" customHeight="1">
+      <x:c r="A53" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B53" s="89"/>
+      <x:c r="C53" s="90"/>
+    </x:row>
+    <x:row r="54" ht="22" customHeight="1">
+      <x:c r="A54" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B54" s="89"/>
+      <x:c r="C54" s="90"/>
+    </x:row>
+    <x:row r="55" ht="22" customHeight="1">
+      <x:c r="A55" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B55" s="89"/>
+      <x:c r="C55" s="90"/>
+    </x:row>
+    <x:row r="56" ht="22" customHeight="1">
+      <x:c r="A56" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B56" s="89"/>
+      <x:c r="C56" s="90"/>
+    </x:row>
+    <x:row r="57" ht="22" customHeight="1">
+      <x:c r="A57" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B57" s="89"/>
+      <x:c r="C57" s="90"/>
+    </x:row>
+    <x:row r="58" ht="22" customHeight="1">
+      <x:c r="A58" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B58" s="89"/>
+      <x:c r="C58" s="90"/>
+    </x:row>
+    <x:row r="59" ht="22" customHeight="1">
+      <x:c r="A59" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B59" s="89"/>
+      <x:c r="C59" s="90"/>
+    </x:row>
+    <x:row r="60" ht="22" customHeight="1">
+      <x:c r="A60" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B60" s="89"/>
+      <x:c r="C60" s="90"/>
+    </x:row>
+    <x:row r="61" ht="22" customHeight="1">
+      <x:c r="A61" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B61" s="89"/>
+      <x:c r="C61" s="90"/>
+    </x:row>
+    <x:row r="62" ht="22" customHeight="1">
+      <x:c r="A62" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B62" s="89"/>
+      <x:c r="C62" s="90"/>
+    </x:row>
+    <x:row r="63" ht="22" customHeight="1">
+      <x:c r="A63" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B63" s="89"/>
+      <x:c r="C63" s="90"/>
+    </x:row>
+    <x:row r="64" ht="22" customHeight="1">
+      <x:c r="A64" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B64" s="89"/>
+      <x:c r="C64" s="90"/>
+    </x:row>
+    <x:row r="65" ht="22" customHeight="1">
+      <x:c r="A65" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B65" s="89"/>
+      <x:c r="C65" s="90"/>
+    </x:row>
+    <x:row r="66" ht="22" customHeight="1">
+      <x:c r="A66" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B66" s="89"/>
+      <x:c r="C66" s="90"/>
+    </x:row>
+    <x:row r="67" ht="22" customHeight="1">
+      <x:c r="A67" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B67" s="89"/>
+      <x:c r="C67" s="90"/>
+    </x:row>
+    <x:row r="68" ht="22" customHeight="1">
+      <x:c r="A68" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B68" s="89"/>
+      <x:c r="C68" s="90"/>
+    </x:row>
+    <x:row r="69" ht="22" customHeight="1">
+      <x:c r="A69" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B69" s="89"/>
+      <x:c r="C69" s="90"/>
+    </x:row>
+    <x:row r="70" ht="22" customHeight="1">
+      <x:c r="A70" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B70" s="89"/>
+      <x:c r="C70" s="90"/>
+    </x:row>
+    <x:row r="71" ht="22" customHeight="1">
+      <x:c r="A71" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B71" s="89"/>
+      <x:c r="C71" s="90"/>
+    </x:row>
+    <x:row r="72" ht="22" customHeight="1">
+      <x:c r="A72" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B72" s="89"/>
+      <x:c r="C72" s="90"/>
+    </x:row>
+    <x:row r="73" ht="22" customHeight="1">
+      <x:c r="A73" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B73" s="89"/>
+      <x:c r="C73" s="90"/>
+    </x:row>
+    <x:row r="74" ht="22" customHeight="1">
+      <x:c r="A74" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B74" s="89"/>
+      <x:c r="C74" s="90"/>
+    </x:row>
+    <x:row r="75" ht="22" customHeight="1">
+      <x:c r="A75" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B75" s="89"/>
+      <x:c r="C75" s="90"/>
+    </x:row>
+    <x:row r="76" ht="22" customHeight="1">
+      <x:c r="A76" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B76" s="89"/>
+      <x:c r="C76" s="90"/>
+    </x:row>
+    <x:row r="77" ht="22" customHeight="1">
+      <x:c r="A77" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B77" s="89"/>
+      <x:c r="C77" s="90"/>
+    </x:row>
+    <x:row r="78" ht="22" customHeight="1">
+      <x:c r="A78" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B78" s="89"/>
+      <x:c r="C78" s="90"/>
+    </x:row>
+    <x:row r="79" ht="22" customHeight="1">
+      <x:c r="A79" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B79" s="89"/>
+      <x:c r="C79" s="90"/>
+    </x:row>
+    <x:row r="80" ht="22" customHeight="1">
+      <x:c r="A80" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B80" s="89"/>
+      <x:c r="C80" s="90"/>
+    </x:row>
+    <x:row r="81" ht="22" customHeight="1">
+      <x:c r="A81" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B81" s="89"/>
+      <x:c r="C81" s="90"/>
+    </x:row>
+    <x:row r="82" ht="22" customHeight="1">
+      <x:c r="A82" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B82" s="89"/>
+      <x:c r="C82" s="90"/>
+    </x:row>
+    <x:row r="83" ht="22" customHeight="1">
+      <x:c r="A83" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B83" s="89"/>
+      <x:c r="C83" s="90"/>
+    </x:row>
+    <x:row r="84" ht="22" customHeight="1">
+      <x:c r="A84" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B84" s="89"/>
+      <x:c r="C84" s="90"/>
+    </x:row>
+    <x:row r="85" ht="22" customHeight="1">
+      <x:c r="A85" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B85" s="89"/>
+      <x:c r="C85" s="90"/>
+    </x:row>
+    <x:row r="86" ht="22" customHeight="1">
+      <x:c r="A86" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B86" s="89"/>
+      <x:c r="C86" s="90"/>
+    </x:row>
+    <x:row r="87" ht="22" customHeight="1">
+      <x:c r="A87" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B87" s="89"/>
+      <x:c r="C87" s="90"/>
+    </x:row>
+    <x:row r="88" ht="22" customHeight="1">
+      <x:c r="A88" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B88" s="89"/>
+      <x:c r="C88" s="90"/>
+    </x:row>
+    <x:row r="89" ht="22" customHeight="1">
+      <x:c r="A89" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B89" s="89"/>
+      <x:c r="C89" s="90"/>
+    </x:row>
+    <x:row r="90" ht="22" customHeight="1">
+      <x:c r="A90" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B90" s="89"/>
+      <x:c r="C90" s="90"/>
+    </x:row>
+    <x:row r="91" ht="22" customHeight="1">
+      <x:c r="A91" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B91" s="89"/>
+      <x:c r="C91" s="90"/>
+    </x:row>
+    <x:row r="92" ht="22" customHeight="1">
+      <x:c r="A92" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B92" s="89"/>
+      <x:c r="C92" s="90"/>
+    </x:row>
+    <x:row r="93" ht="22" customHeight="1">
+      <x:c r="A93" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B93" s="89"/>
+      <x:c r="C93" s="90"/>
+    </x:row>
+    <x:row r="94" ht="22" customHeight="1">
+      <x:c r="A94" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B94" s="89"/>
+      <x:c r="C94" s="90"/>
+    </x:row>
+    <x:row r="95" ht="22" customHeight="1">
+      <x:c r="A95" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B95" s="89"/>
+      <x:c r="C95" s="90"/>
+    </x:row>
+    <x:row r="96" ht="22" customHeight="1">
+      <x:c r="A96" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B96" s="89"/>
+      <x:c r="C96" s="90"/>
+    </x:row>
+    <x:row r="97" ht="22" customHeight="1">
+      <x:c r="A97" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B97" s="89"/>
+      <x:c r="C97" s="90"/>
+    </x:row>
+    <x:row r="98" ht="22" customHeight="1">
+      <x:c r="A98" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B98" s="89"/>
+      <x:c r="C98" s="90"/>
+    </x:row>
+    <x:row r="99" ht="22" customHeight="1">
+      <x:c r="A99" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B99" s="89"/>
+      <x:c r="C99" s="90"/>
+    </x:row>
+    <x:row r="100" ht="22" customHeight="1">
+      <x:c r="A100" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B100" s="89"/>
+      <x:c r="C100" s="90"/>
+    </x:row>
+    <x:row r="101" ht="22" customHeight="1">
+      <x:c r="A101" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B101" s="89"/>
+      <x:c r="C101" s="90"/>
+    </x:row>
+    <x:row r="102" ht="22" customHeight="1">
+      <x:c r="A102" s="88" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B102" s="89"/>
+      <x:c r="C102" s="90"/>
+    </x:row>
+    <x:row r="103" ht="22" customHeight="1">
+      <x:c r="A103" s="91" t="str">
+        <x:v>Esterno</x:v>
+      </x:c>
+      <x:c r="B103" s="92"/>
+      <x:c r="C103" s="93"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:C1"/>
+    <x:mergeCell ref="A2:C2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R49d14cd067fb4f9a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6830,8 +7731,8 @@
       <x:c r="B8" s="74" t="s">
         <x:v>67</x:v>
       </x:c>
-      <x:c r="C8" s="74" t="s">
-        <x:v>68</x:v>
+      <x:c r="C8" s="74" t="str">
+        <x:v>Registra ogni affidatario in Affidamenti_Patch. Per colleghi o amici, aggiungi prima il nome in Venditori_Affidatari; poi selezionalo nei menu di affidamenti e vendite.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="20" customHeight="1">
@@ -7575,7 +8476,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R07922a4f70bf4b27"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7562d3e5bc974a38"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11067,7 +11968,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R45ad750f3dfb4a8f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R509b329d3f0f47b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -18655,12 +19556,12 @@
   </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="L4:L303">
-      <x:formula1>'Persone_Quote'!$B$4:$B$18</x:formula1>
+      <x:formula1>'Venditori_Affidatari'!$B$4:$B$103</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra8e61bf009e94c5f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rddf3658dfe98453a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21144,7 +22045,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b002e42db17492a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra6137faf510e4799"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21629,7 +22530,7 @@
     </x:cfRule>
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra3b429e6e9b24d13"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R762d04446f30420e"/>
 </x:worksheet>
 </file>
 

</xml_diff>